<commit_message>
fix spinbox issue of artifacts
</commit_message>
<xml_diff>
--- a/master_workbook.xlsx
+++ b/master_workbook.xlsx
@@ -10,15 +10,14 @@
     <sheet name="digestion_page" sheetId="1" r:id="rId1"/>
     <sheet name="200120001" sheetId="2" r:id="rId2"/>
     <sheet name="200120002" sheetId="3" r:id="rId3"/>
-    <sheet name="200120003" sheetId="4" r:id="rId4"/>
-    <sheet name="formula_page" sheetId="5" r:id="rId5"/>
+    <sheet name="formula_page" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="77">
   <si>
     <t>Date:</t>
   </si>
@@ -26,16 +25,16 @@
     <t>Request ID:</t>
   </si>
   <si>
-    <t>100048665</t>
+    <t>TEST</t>
   </si>
   <si>
     <t>Microwave</t>
   </si>
   <si>
-    <t>Element(s)</t>
-  </si>
-  <si>
-    <t>Al, Ca</t>
+    <t>Analyte(s)</t>
+  </si>
+  <si>
+    <t>Mg</t>
   </si>
   <si>
     <t>SOP#</t>
@@ -89,13 +88,31 @@
     <t>200120002_2</t>
   </si>
   <si>
-    <t>200120003_1</t>
-  </si>
-  <si>
-    <t>200120003_2</t>
-  </si>
-  <si>
-    <t>Al ICP analysis</t>
+    <t>Mn</t>
+  </si>
+  <si>
+    <t>Katanax</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Kr</t>
+  </si>
+  <si>
+    <t>Hotplate</t>
+  </si>
+  <si>
+    <t>Hf</t>
+  </si>
+  <si>
+    <t>Cocktail</t>
+  </si>
+  <si>
+    <t>Hs</t>
+  </si>
+  <si>
+    <t>Mg ICP analysis</t>
   </si>
   <si>
     <t>sample</t>
@@ -107,49 +124,118 @@
     <t>conc. [mg/L]</t>
   </si>
   <si>
-    <t>Al_ppm</t>
-  </si>
-  <si>
-    <t>%Al</t>
-  </si>
-  <si>
-    <t>al result:</t>
-  </si>
-  <si>
-    <t>al oxide factor:</t>
-  </si>
-  <si>
-    <t>al oxide result:</t>
-  </si>
-  <si>
-    <t>al lot:</t>
-  </si>
-  <si>
-    <t>Ca ICP analysis</t>
-  </si>
-  <si>
-    <t>Ca_ppm</t>
-  </si>
-  <si>
-    <t>%Ca</t>
-  </si>
-  <si>
-    <t>ca result:</t>
-  </si>
-  <si>
-    <t>ca oxide factor:</t>
-  </si>
-  <si>
-    <t>ca oxide result:</t>
-  </si>
-  <si>
-    <t>ca lot:</t>
-  </si>
-  <si>
-    <t>Manufacturer: Assurance, 27-171ALT exp: 2026-07-30</t>
-  </si>
-  <si>
-    <t>Manufacturer: Assurance, 28-35CAY exp: 2026-10-30</t>
+    <t>Mg_ppm</t>
+  </si>
+  <si>
+    <t>%Mg</t>
+  </si>
+  <si>
+    <t>mg result:</t>
+  </si>
+  <si>
+    <t>mg oxide factor:</t>
+  </si>
+  <si>
+    <t>mg oxide result:</t>
+  </si>
+  <si>
+    <t>mg lot:</t>
+  </si>
+  <si>
+    <t>Mn ICP analysis</t>
+  </si>
+  <si>
+    <t>Mn_ppm</t>
+  </si>
+  <si>
+    <t>%Mn</t>
+  </si>
+  <si>
+    <t>mn result:</t>
+  </si>
+  <si>
+    <t>mn oxide factor:</t>
+  </si>
+  <si>
+    <t>mn oxide result:</t>
+  </si>
+  <si>
+    <t>mn lot:</t>
+  </si>
+  <si>
+    <t>K ICP analysis</t>
+  </si>
+  <si>
+    <t>K_ppm</t>
+  </si>
+  <si>
+    <t>%K</t>
+  </si>
+  <si>
+    <t>k result:</t>
+  </si>
+  <si>
+    <t>k oxide factor:</t>
+  </si>
+  <si>
+    <t>k oxide result:</t>
+  </si>
+  <si>
+    <t>k lot:</t>
+  </si>
+  <si>
+    <t>Kr ICP analysis</t>
+  </si>
+  <si>
+    <t>Kr_ppm</t>
+  </si>
+  <si>
+    <t>%Kr</t>
+  </si>
+  <si>
+    <t>kr result:</t>
+  </si>
+  <si>
+    <t>kr lot:</t>
+  </si>
+  <si>
+    <t>Hf ICP analysis</t>
+  </si>
+  <si>
+    <t>Hf_ppm</t>
+  </si>
+  <si>
+    <t>%Hf</t>
+  </si>
+  <si>
+    <t>hf result:</t>
+  </si>
+  <si>
+    <t>hf oxide factor:</t>
+  </si>
+  <si>
+    <t>hf oxide result:</t>
+  </si>
+  <si>
+    <t>hf lot:</t>
+  </si>
+  <si>
+    <t>Hs ICP analysis</t>
+  </si>
+  <si>
+    <t>Hs_ppm</t>
+  </si>
+  <si>
+    <t>%Hs</t>
+  </si>
+  <si>
+    <t>hs result:</t>
+  </si>
+  <si>
+    <t>hs lot:</t>
+  </si>
+  <si>
+    <t>Manufacturer: Assurance, 28-6KY exp: 2026-08-30</t>
   </si>
   <si>
     <t>Note(s):</t>
@@ -591,10 +677,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.140625" bestFit="1" customWidth="1"/>
@@ -606,7 +692,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46197</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -751,50 +837,490 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:5">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="6"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:5">
       <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="6"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="6"/>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:5">
       <c r="A20" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="6"/>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="5" t="s">
+    <row r="23" spans="1:5">
+      <c r="A23" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="6"/>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="5" t="s">
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="6">
+        <v>15</v>
+      </c>
+      <c r="B31" s="6">
+        <v>1200</v>
+      </c>
+      <c r="C31" s="6">
+        <v>180</v>
+      </c>
+      <c r="D31" s="6">
+        <v>65</v>
+      </c>
+      <c r="E31" s="6">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="6">
+        <v>15</v>
+      </c>
+      <c r="B32" s="6">
+        <v>1500</v>
+      </c>
+      <c r="C32" s="6">
+        <v>240</v>
+      </c>
+      <c r="D32" s="6">
+        <v>65</v>
+      </c>
+      <c r="E32" s="6">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" s="8"/>
+      <c r="C35" s="6"/>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="8"/>
+      <c r="C36" s="6"/>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B37" s="8"/>
+      <c r="C37" s="6"/>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B38" s="8"/>
+      <c r="C38" s="6"/>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="6"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C42" s="6"/>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6"/>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B46" s="8"/>
+      <c r="C46" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47" s="8"/>
+      <c r="C47" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B48" s="8"/>
+      <c r="C48" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B49" s="8"/>
+      <c r="C49" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C53" s="6"/>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6"/>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" s="8"/>
+      <c r="C57" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" s="8"/>
+      <c r="C58" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B59" s="8"/>
+      <c r="C59" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" s="8"/>
+      <c r="C60" s="6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C64" s="6"/>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" s="6"/>
+      <c r="C65" s="6"/>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B68" s="8"/>
+      <c r="C68" s="6"/>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B69" s="8"/>
+      <c r="C69" s="6"/>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B70" s="8"/>
+      <c r="C70" s="6"/>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B71" s="8"/>
+      <c r="C71" s="6"/>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C75" s="6"/>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B76" s="6"/>
+      <c r="C76" s="6"/>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B77" s="6"/>
+      <c r="C77" s="6"/>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B79" s="8"/>
+      <c r="C79" s="6"/>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B80" s="8"/>
+      <c r="C80" s="6"/>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B81" s="8"/>
+      <c r="C81" s="6"/>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B82" s="8"/>
+      <c r="C82" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="30">
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B7:E7"/>
@@ -802,6 +1328,29 @@
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B11:E11"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="A63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="A74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B77:C77"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -809,14 +1358,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="17" width="7.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="59" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -824,7 +1373,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46197</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -837,25 +1386,25 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -920,7 +1469,7 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="13">
@@ -930,7 +1479,7 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="14">
@@ -940,14 +1489,14 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="12" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="12" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="14">
@@ -957,37 +1506,35 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="12" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B14" s="12"/>
-      <c r="C14" s="15" t="s">
-        <v>42</v>
-      </c>
+      <c r="C14" s="15"/>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B16" s="3"/>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1008,11 +1555,11 @@
         <v>0</v>
       </c>
       <c r="G18" s="11">
-        <f>digestion_page!B17</f>
+        <f>digestion_page!B35</f>
         <v>0</v>
       </c>
       <c r="H18" s="11">
-        <f>digestion_page!C17</f>
+        <f>digestion_page!C35</f>
         <v>0</v>
       </c>
       <c r="I18" s="11">
@@ -1038,11 +1585,11 @@
         <v>0</v>
       </c>
       <c r="G19" s="11">
-        <f>digestion_page!B18</f>
+        <f>digestion_page!B36</f>
         <v>0</v>
       </c>
       <c r="H19" s="11">
-        <f>digestion_page!C18</f>
+        <f>digestion_page!C36</f>
         <v>0</v>
       </c>
       <c r="I19" s="11">
@@ -1052,7 +1599,7 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="12" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="13">
@@ -1062,7 +1609,7 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="12" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="14">
@@ -1072,14 +1619,14 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="12" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="12" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="14">
@@ -1089,39 +1636,525 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="12" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B25" s="12"/>
-      <c r="C25" s="15" t="s">
-        <v>43</v>
-      </c>
+      <c r="C25" s="15"/>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
       <c r="F25" s="15"/>
     </row>
     <row r="27" spans="1:9">
-      <c r="B27" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
+      <c r="A27" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="3"/>
     </row>
     <row r="28" spans="1:9">
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
+      <c r="A28" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="29" spans="1:9">
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="A29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10">
+        <f>((C29)*(H29)*(I29))/(G29*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="10">
+        <f>D29/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="11">
+        <f>digestion_page!B46</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="11">
+        <f>digestion_page!C46</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="11">
+        <f>(LEFT(B29,FIND("/",B29)-1)/RIGHT(B29,LEN(B29)-FIND("/", B29)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="10">
+        <f>((C30)*(H30)*(I30))/(G30*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="10">
+        <f>D30/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="11">
+        <f>digestion_page!B47</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="11">
+        <f>digestion_page!C47</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="11">
+        <f>(LEFT(B30,FIND("/",B30)-1)/RIGHT(B30,LEN(B30)-FIND("/", B30)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="12"/>
+      <c r="C32" s="13">
+        <f>AVERAGE(D29:D30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="12"/>
+      <c r="C33" s="14">
+        <f>AVERAGE(E29:E30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="12"/>
+      <c r="C34" s="3"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="12"/>
+      <c r="C35" s="14">
+        <f>AVERAGE(E29:E30)*(C34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="12"/>
+      <c r="C36" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" s="3"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B40" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="9"/>
+      <c r="D40" s="10">
+        <f>((C40)*(H40)*(I40))/(G40*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="10">
+        <f>D40/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="11">
+        <f>digestion_page!B57</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="11">
+        <f>digestion_page!C57</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="11">
+        <f>(LEFT(B40,FIND("/",B40)-1)/RIGHT(B40,LEN(B40)-FIND("/", B40)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="9"/>
+      <c r="D41" s="10">
+        <f>((C41)*(H41)*(I41))/(G41*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="10">
+        <f>D41/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="11">
+        <f>digestion_page!B58</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="11">
+        <f>digestion_page!C58</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="11">
+        <f>(LEFT(B41,FIND("/",B41)-1)/RIGHT(B41,LEN(B41)-FIND("/", B41)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" s="12"/>
+      <c r="C43" s="13">
+        <f>AVERAGE(D40:D41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="12"/>
+      <c r="C44" s="14">
+        <f>AVERAGE(E40:E41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B45" s="12"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="3"/>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B49" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C49" s="9"/>
+      <c r="D49" s="10">
+        <f>((C49)*(H49)*(I49))/(G49*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E49" s="10">
+        <f>D49/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G49" s="11">
+        <f>digestion_page!B68</f>
+        <v>0</v>
+      </c>
+      <c r="H49" s="11">
+        <f>digestion_page!C68</f>
+        <v>0</v>
+      </c>
+      <c r="I49" s="11">
+        <f>(LEFT(B49,FIND("/",B49)-1)/RIGHT(B49,LEN(B49)-FIND("/", B49)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B50" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C50" s="9"/>
+      <c r="D50" s="10">
+        <f>((C50)*(H50)*(I50))/(G50*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E50" s="10">
+        <f>D50/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G50" s="11">
+        <f>digestion_page!B69</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="11">
+        <f>digestion_page!C69</f>
+        <v>0</v>
+      </c>
+      <c r="I50" s="11">
+        <f>(LEFT(B50,FIND("/",B50)-1)/RIGHT(B50,LEN(B50)-FIND("/", B50)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B52" s="12"/>
+      <c r="C52" s="13">
+        <f>AVERAGE(D49:D50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B53" s="12"/>
+      <c r="C53" s="14">
+        <f>AVERAGE(E49:E50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B54" s="12"/>
+      <c r="C54" s="3"/>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55" s="12"/>
+      <c r="C55" s="14">
+        <f>AVERAGE(E49:E50)*(C54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="12"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B58" s="3"/>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B60" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C60" s="9"/>
+      <c r="D60" s="10">
+        <f>((C60)*(H60)*(I60))/(G60*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E60" s="10">
+        <f>D60/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G60" s="11">
+        <f>digestion_page!B79</f>
+        <v>0</v>
+      </c>
+      <c r="H60" s="11">
+        <f>digestion_page!C79</f>
+        <v>0</v>
+      </c>
+      <c r="I60" s="11">
+        <f>(LEFT(B60,FIND("/",B60)-1)/RIGHT(B60,LEN(B60)-FIND("/", B60)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9">
+      <c r="A61" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B61" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C61" s="9"/>
+      <c r="D61" s="10">
+        <f>((C61)*(H61)*(I61))/(G61*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E61" s="10">
+        <f>D61/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G61" s="11">
+        <f>digestion_page!B80</f>
+        <v>0</v>
+      </c>
+      <c r="H61" s="11">
+        <f>digestion_page!C80</f>
+        <v>0</v>
+      </c>
+      <c r="I61" s="11">
+        <f>(LEFT(B61,FIND("/",B61)-1)/RIGHT(B61,LEN(B61)-FIND("/", B61)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="A63" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B63" s="12"/>
+      <c r="C63" s="13">
+        <f>AVERAGE(D60:D61)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9">
+      <c r="A64" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" s="12"/>
+      <c r="C64" s="14">
+        <f>AVERAGE(E60:E61)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B65" s="12"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="15"/>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="B67" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="39">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
@@ -1136,7 +2169,31 @@
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C25:F25"/>
-    <mergeCell ref="C27:F29"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="C56:F56"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="C65:F65"/>
+    <mergeCell ref="C67:F69"/>
   </mergeCells>
   <conditionalFormatting sqref="C14:F14">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
@@ -1148,20 +2205,40 @@
       <formula>LEN(TRIM(C25))=0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C36:F36">
+    <cfRule type="containsBlanks" dxfId="0" priority="3">
+      <formula>LEN(TRIM(C36))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C45:F45">
+    <cfRule type="containsBlanks" dxfId="0" priority="4">
+      <formula>LEN(TRIM(C45))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C56:F56">
+    <cfRule type="containsBlanks" dxfId="0" priority="5">
+      <formula>LEN(TRIM(C56))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C65:F65">
+    <cfRule type="containsBlanks" dxfId="0" priority="6">
+      <formula>LEN(TRIM(C65))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="17" width="7.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="59" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1169,7 +2246,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46197</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1182,25 +2259,25 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1265,7 +2342,7 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="13">
@@ -1275,7 +2352,7 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="14">
@@ -1285,14 +2362,14 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="12" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="12" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="14">
@@ -1302,37 +2379,35 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="12" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B14" s="12"/>
-      <c r="C14" s="15" t="s">
-        <v>42</v>
-      </c>
+      <c r="C14" s="15"/>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B16" s="3"/>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1353,11 +2428,11 @@
         <v>0</v>
       </c>
       <c r="G18" s="11">
-        <f>digestion_page!B19</f>
+        <f>digestion_page!B37</f>
         <v>0</v>
       </c>
       <c r="H18" s="11">
-        <f>digestion_page!C19</f>
+        <f>digestion_page!C37</f>
         <v>0</v>
       </c>
       <c r="I18" s="11">
@@ -1383,11 +2458,11 @@
         <v>0</v>
       </c>
       <c r="G19" s="11">
-        <f>digestion_page!B20</f>
+        <f>digestion_page!B38</f>
         <v>0</v>
       </c>
       <c r="H19" s="11">
-        <f>digestion_page!C20</f>
+        <f>digestion_page!C38</f>
         <v>0</v>
       </c>
       <c r="I19" s="11">
@@ -1397,7 +2472,7 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="12" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="13">
@@ -1407,7 +2482,7 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="12" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="14">
@@ -1417,14 +2492,14 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="12" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="12" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="14">
@@ -1434,39 +2509,525 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="12" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B25" s="12"/>
-      <c r="C25" s="15" t="s">
-        <v>43</v>
-      </c>
+      <c r="C25" s="15"/>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
       <c r="F25" s="15"/>
     </row>
     <row r="27" spans="1:9">
-      <c r="B27" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
+      <c r="A27" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="3"/>
     </row>
     <row r="28" spans="1:9">
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
+      <c r="A28" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="29" spans="1:9">
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="A29" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10">
+        <f>((C29)*(H29)*(I29))/(G29*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="10">
+        <f>D29/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="11">
+        <f>digestion_page!B48</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="11">
+        <f>digestion_page!C48</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="11">
+        <f>(LEFT(B29,FIND("/",B29)-1)/RIGHT(B29,LEN(B29)-FIND("/", B29)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="10">
+        <f>((C30)*(H30)*(I30))/(G30*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="10">
+        <f>D30/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="11">
+        <f>digestion_page!B49</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="11">
+        <f>digestion_page!C49</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="11">
+        <f>(LEFT(B30,FIND("/",B30)-1)/RIGHT(B30,LEN(B30)-FIND("/", B30)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="12"/>
+      <c r="C32" s="13">
+        <f>AVERAGE(D29:D30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="12"/>
+      <c r="C33" s="14">
+        <f>AVERAGE(E29:E30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="12"/>
+      <c r="C34" s="3"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="12"/>
+      <c r="C35" s="14">
+        <f>AVERAGE(E29:E30)*(C34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="12"/>
+      <c r="C36" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" s="3"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B40" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="9"/>
+      <c r="D40" s="10">
+        <f>((C40)*(H40)*(I40))/(G40*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="10">
+        <f>D40/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="11">
+        <f>digestion_page!B59</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="11">
+        <f>digestion_page!C59</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="11">
+        <f>(LEFT(B40,FIND("/",B40)-1)/RIGHT(B40,LEN(B40)-FIND("/", B40)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="9"/>
+      <c r="D41" s="10">
+        <f>((C41)*(H41)*(I41))/(G41*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="10">
+        <f>D41/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="11">
+        <f>digestion_page!B60</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="11">
+        <f>digestion_page!C60</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="11">
+        <f>(LEFT(B41,FIND("/",B41)-1)/RIGHT(B41,LEN(B41)-FIND("/", B41)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" s="12"/>
+      <c r="C43" s="13">
+        <f>AVERAGE(D40:D41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="12"/>
+      <c r="C44" s="14">
+        <f>AVERAGE(E40:E41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B45" s="12"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="3"/>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B49" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C49" s="9"/>
+      <c r="D49" s="10">
+        <f>((C49)*(H49)*(I49))/(G49*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E49" s="10">
+        <f>D49/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G49" s="11">
+        <f>digestion_page!B70</f>
+        <v>0</v>
+      </c>
+      <c r="H49" s="11">
+        <f>digestion_page!C70</f>
+        <v>0</v>
+      </c>
+      <c r="I49" s="11">
+        <f>(LEFT(B49,FIND("/",B49)-1)/RIGHT(B49,LEN(B49)-FIND("/", B49)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B50" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C50" s="9"/>
+      <c r="D50" s="10">
+        <f>((C50)*(H50)*(I50))/(G50*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E50" s="10">
+        <f>D50/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G50" s="11">
+        <f>digestion_page!B71</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="11">
+        <f>digestion_page!C71</f>
+        <v>0</v>
+      </c>
+      <c r="I50" s="11">
+        <f>(LEFT(B50,FIND("/",B50)-1)/RIGHT(B50,LEN(B50)-FIND("/", B50)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B52" s="12"/>
+      <c r="C52" s="13">
+        <f>AVERAGE(D49:D50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B53" s="12"/>
+      <c r="C53" s="14">
+        <f>AVERAGE(E49:E50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B54" s="12"/>
+      <c r="C54" s="3"/>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55" s="12"/>
+      <c r="C55" s="14">
+        <f>AVERAGE(E49:E50)*(C54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="12"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B58" s="3"/>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B60" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C60" s="9"/>
+      <c r="D60" s="10">
+        <f>((C60)*(H60)*(I60))/(G60*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E60" s="10">
+        <f>D60/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G60" s="11">
+        <f>digestion_page!B81</f>
+        <v>0</v>
+      </c>
+      <c r="H60" s="11">
+        <f>digestion_page!C81</f>
+        <v>0</v>
+      </c>
+      <c r="I60" s="11">
+        <f>(LEFT(B60,FIND("/",B60)-1)/RIGHT(B60,LEN(B60)-FIND("/", B60)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9">
+      <c r="A61" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B61" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C61" s="9"/>
+      <c r="D61" s="10">
+        <f>((C61)*(H61)*(I61))/(G61*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E61" s="10">
+        <f>D61/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G61" s="11">
+        <f>digestion_page!B82</f>
+        <v>0</v>
+      </c>
+      <c r="H61" s="11">
+        <f>digestion_page!C82</f>
+        <v>0</v>
+      </c>
+      <c r="I61" s="11">
+        <f>(LEFT(B61,FIND("/",B61)-1)/RIGHT(B61,LEN(B61)-FIND("/", B61)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="A63" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B63" s="12"/>
+      <c r="C63" s="13">
+        <f>AVERAGE(D60:D61)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9">
+      <c r="A64" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" s="12"/>
+      <c r="C64" s="14">
+        <f>AVERAGE(E60:E61)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B65" s="12"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="15"/>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="B67" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="39">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
@@ -1481,7 +3042,31 @@
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C25:F25"/>
-    <mergeCell ref="C27:F29"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="C56:F56"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="C65:F65"/>
+    <mergeCell ref="C67:F69"/>
   </mergeCells>
   <conditionalFormatting sqref="C14:F14">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
@@ -1493,356 +3078,31 @@
       <formula>LEN(TRIM(C25))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="17" width="7.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2">
-        <v>46197</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="6">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="10">
-        <f>((C7)*(H7)*(I7))/(G7*1)</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="10">
-        <f>D7/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="11">
-        <f>digestion_page!B21</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="11">
-        <f>digestion_page!C21</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="11">
-        <f>(LEFT(B7,FIND("/",B7)-1)/RIGHT(B7,LEN(B7)-FIND("/", B7)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="6">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="10">
-        <f>((C8)*(H8)*(I8))/(G8*1)</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="10">
-        <f>D8/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="11">
-        <f>digestion_page!B22</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="11">
-        <f>digestion_page!C22</f>
-        <v>0</v>
-      </c>
-      <c r="I8" s="11">
-        <f>(LEFT(B8,FIND("/",B8)-1)/RIGHT(B8,LEN(B8)-FIND("/", B8)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13">
-        <f>AVERAGE(D7:D8)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="14">
-        <f>AVERAGE(E7:E8)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="3"/>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="14">
-        <f>AVERAGE(E7:E8)*(C12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="3"/>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="6">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="10">
-        <f>((C18)*(H18)*(I18))/(G18*1)</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="10">
-        <f>D18/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="11">
-        <f>digestion_page!B21</f>
-        <v>0</v>
-      </c>
-      <c r="H18" s="11">
-        <f>digestion_page!C21</f>
-        <v>0</v>
-      </c>
-      <c r="I18" s="11">
-        <f>(LEFT(B18,FIND("/",B18)-1)/RIGHT(B18,LEN(B18)-FIND("/", B18)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="6">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="10">
-        <f>((C19)*(H19)*(I19))/(G19*1)</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="10">
-        <f>D19/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G19" s="11">
-        <f>digestion_page!B22</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="11">
-        <f>digestion_page!C22</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="11">
-        <f>(LEFT(B19,FIND("/",B19)-1)/RIGHT(B19,LEN(B19)-FIND("/", B19)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13">
-        <f>AVERAGE(D18:D19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="12"/>
-      <c r="C22" s="14">
-        <f>AVERAGE(E18:E19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="3"/>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="12"/>
-      <c r="C24" s="14">
-        <f>AVERAGE(E18:E19)*(C23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="B27" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-    </row>
-  </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="C27:F29"/>
-  </mergeCells>
-  <conditionalFormatting sqref="C14:F14">
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(C14))=0</formula>
+  <conditionalFormatting sqref="C36:F36">
+    <cfRule type="containsBlanks" dxfId="0" priority="3">
+      <formula>LEN(TRIM(C36))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C25:F25">
-    <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(C25))=0</formula>
+  <conditionalFormatting sqref="C45:F45">
+    <cfRule type="containsBlanks" dxfId="0" priority="4">
+      <formula>LEN(TRIM(C45))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C56:F56">
+    <cfRule type="containsBlanks" dxfId="0" priority="5">
+      <formula>LEN(TRIM(C56))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C65:F65">
+    <cfRule type="containsBlanks" dxfId="0" priority="6">
+      <formula>LEN(TRIM(C65))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1852,17 +3112,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="17" t="s">
-        <v>45</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="17" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="17" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates are attached to live app.
</commit_message>
<xml_diff>
--- a/master_workbook.xlsx
+++ b/master_workbook.xlsx
@@ -8,29 +8,160 @@
   </bookViews>
   <sheets>
     <sheet name="digestion_page" sheetId="1" r:id="rId1"/>
-    <sheet name="formula_page" sheetId="2" r:id="rId2"/>
+    <sheet name="200120001" sheetId="2" r:id="rId2"/>
+    <sheet name="200120002" sheetId="3" r:id="rId3"/>
+    <sheet name="formula_page" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="43">
   <si>
     <t>Date:</t>
   </si>
   <si>
     <t>Request ID:</t>
+  </si>
+  <si>
+    <t>100048600</t>
+  </si>
+  <si>
+    <t>Hotplate</t>
+  </si>
+  <si>
+    <t>Analyte(s)</t>
+  </si>
+  <si>
+    <t>Mn</t>
+  </si>
+  <si>
+    <t>SOP#</t>
+  </si>
+  <si>
+    <t>Cocktail</t>
+  </si>
+  <si>
+    <t>sample(s)</t>
+  </si>
+  <si>
+    <t>weight (g)</t>
+  </si>
+  <si>
+    <t>volume (mL)</t>
+  </si>
+  <si>
+    <t>200120001_1</t>
+  </si>
+  <si>
+    <t>200120001_2</t>
+  </si>
+  <si>
+    <t>200120002_1</t>
+  </si>
+  <si>
+    <t>200120002_2</t>
+  </si>
+  <si>
+    <t>LOI temp:</t>
+  </si>
+  <si>
+    <t>sample</t>
+  </si>
+  <si>
+    <t>crucible (g)</t>
+  </si>
+  <si>
+    <t>crucible + sample (g)</t>
+  </si>
+  <si>
+    <t>LOI (%)</t>
+  </si>
+  <si>
+    <t>correction</t>
+  </si>
+  <si>
+    <t>200120001</t>
+  </si>
+  <si>
+    <t>Mn ICP analysis</t>
+  </si>
+  <si>
+    <t>Dilution</t>
+  </si>
+  <si>
+    <t>conc. [mg/L]</t>
+  </si>
+  <si>
+    <t>Mn_ppm [dried]</t>
+  </si>
+  <si>
+    <t>%Mn [dried]</t>
+  </si>
+  <si>
+    <t>mn result:</t>
+  </si>
+  <si>
+    <t>mn oxide factor:</t>
+  </si>
+  <si>
+    <t>mn oxide result:</t>
+  </si>
+  <si>
+    <t>mn lot:</t>
+  </si>
+  <si>
+    <t>Note(s):</t>
+  </si>
+  <si>
+    <t>200120002</t>
+  </si>
+  <si>
+    <t>ppm M+ = [conc.][volume][dilution]/[weight]</t>
+  </si>
+  <si>
+    <t>%M+ = [conc.][volume][dilution]/([weight]*10,000)</t>
+  </si>
+  <si>
+    <t>%MO = [oxide factor]*%M+</t>
+  </si>
+  <si>
+    <t>A = crucible</t>
+  </si>
+  <si>
+    <t>B = crucible + sample</t>
+  </si>
+  <si>
+    <t>C = crucible + sample after drying</t>
+  </si>
+  <si>
+    <t>%LOI = ([B-A]-[C-A])/(B-A)*100%</t>
+  </si>
+  <si>
+    <t>ppm M+  [dried] = ppm M+/([1-(%LOI)/100])</t>
+  </si>
+  <si>
+    <t>%M+  [dried] = %M+/([1-(%LOI)/100])</t>
+  </si>
+  <si>
+    <t>%MO [dried] = %MO/([1-(%LOI)/100])</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="######&quot; °C&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="0.00&quot; ppm&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.00&quot; %&quot;"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -46,6 +177,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -55,7 +210,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -63,11 +218,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -78,11 +248,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -372,33 +574,667 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46206</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="6"/>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="7.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="9"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="5">
+        <f>"after "&amp;B5&amp;" °C"</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="10">
+        <f>(((C7-B7)-(D7-B7))/(C7-B7))*100</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="7">
+        <f>1-(E7/100)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="10">
+        <f>((C11)*(H11)*(I11))/(G11*$F$7)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="10">
+        <f>D11/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <f>digestion_page!B10</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="12">
+        <f>digestion_page!C10</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="12">
+        <f>(LEFT(B11,FIND("/",B11)-1)/RIGHT(B11,LEN(B11)-FIND("/", B11)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="11"/>
+      <c r="D12" s="10">
+        <f>((C12)*(H12)*(I12))/(G12*$F$7)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="10">
+        <f>D12/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="12">
+        <f>digestion_page!B11</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="12">
+        <f>digestion_page!C11</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="12">
+        <f>(LEFT(B12,FIND("/",B12)-1)/RIGHT(B12,LEN(B12)-FIND("/", B12)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="13">
+        <f>AVERAGE(D11:D12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="8"/>
+      <c r="C15" s="14">
+        <f>AVERAGE(E11:E12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="14">
+        <f>AVERAGE(E11:E12)*(C16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="8"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="B20" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C20:F22"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(B5))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18:F18">
+    <cfRule type="containsBlanks" dxfId="0" priority="2">
+      <formula>LEN(TRIM(C18))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="7.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="9"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="5">
+        <f>"after "&amp;B5&amp;" °C"</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="10">
+        <f>(((C7-B7)-(D7-B7))/(C7-B7))*100</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="7">
+        <f>1-(E7/100)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="10">
+        <f>((C11)*(H11)*(I11))/(G11*$F$7)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="10">
+        <f>D11/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <f>digestion_page!B12</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="12">
+        <f>digestion_page!C12</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="12">
+        <f>(LEFT(B11,FIND("/",B11)-1)/RIGHT(B11,LEN(B11)-FIND("/", B11)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="11"/>
+      <c r="D12" s="10">
+        <f>((C12)*(H12)*(I12))/(G12*$F$7)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="10">
+        <f>D12/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="12">
+        <f>digestion_page!B13</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="12">
+        <f>digestion_page!C13</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="12">
+        <f>(LEFT(B12,FIND("/",B12)-1)/RIGHT(B12,LEN(B12)-FIND("/", B12)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="13">
+        <f>AVERAGE(D11:D12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="8"/>
+      <c r="C15" s="14">
+        <f>AVERAGE(E11:E12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="14">
+        <f>AVERAGE(E11:E12)*(C16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="8"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="B20" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C20:F22"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(B5))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18:F18">
+    <cfRule type="containsBlanks" dxfId="0" priority="2">
+      <formula>LEN(TRIM(C18))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="46.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="17" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
still has a bug when it comes to titrations
</commit_message>
<xml_diff>
--- a/master_workbook.xlsx
+++ b/master_workbook.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="39">
   <si>
     <t>Date:</t>
   </si>
@@ -24,46 +24,22 @@
     <t>Request ID:</t>
   </si>
   <si>
-    <t>100048800</t>
-  </si>
-  <si>
-    <t>Microwave</t>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>Hotplate</t>
   </si>
   <si>
     <t>Analyte(s)</t>
   </si>
   <si>
-    <t>Ti</t>
+    <t>Al</t>
   </si>
   <si>
     <t>SOP#</t>
   </si>
   <si>
-    <t>Acid Cocktail</t>
-  </si>
-  <si>
-    <t>Rack</t>
-  </si>
-  <si>
-    <t>Vessel</t>
-  </si>
-  <si>
-    <t>Stir</t>
-  </si>
-  <si>
-    <t>Time (min)</t>
-  </si>
-  <si>
-    <t>Power (W)</t>
-  </si>
-  <si>
-    <t>T1 (°C)</t>
-  </si>
-  <si>
-    <t>T2 (°C)</t>
-  </si>
-  <si>
-    <t>P (bar)</t>
+    <t>Cocktail</t>
   </si>
   <si>
     <t>sample(s)</t>
@@ -81,52 +57,70 @@
     <t>200120001_2</t>
   </si>
   <si>
-    <t>Hotplate</t>
-  </si>
-  <si>
-    <t>Cr2O3</t>
-  </si>
-  <si>
-    <t>Cocktail</t>
-  </si>
-  <si>
-    <t>Cr2O3 titration analysis</t>
+    <t>Al, Ca</t>
+  </si>
+  <si>
+    <t>200120001_3</t>
+  </si>
+  <si>
+    <t>200120001_4</t>
+  </si>
+  <si>
+    <t>Ca</t>
+  </si>
+  <si>
+    <t>200120001_5</t>
+  </si>
+  <si>
+    <t>200120001_6</t>
+  </si>
+  <si>
+    <t>Al ICP analysis</t>
   </si>
   <si>
     <t>sample</t>
   </si>
   <si>
-    <t>titrant_volume (mL)</t>
-  </si>
-  <si>
-    <t>%Cr2O3</t>
-  </si>
-  <si>
-    <t>FAS:</t>
-  </si>
-  <si>
-    <t>cr2o3 result:</t>
-  </si>
-  <si>
-    <t>Ti ICP analysis</t>
-  </si>
-  <si>
     <t>Dilution</t>
   </si>
   <si>
     <t>conc. [mg/L]</t>
   </si>
   <si>
-    <t>Ti_ppm</t>
-  </si>
-  <si>
-    <t>%Ti</t>
-  </si>
-  <si>
-    <t>ti result:</t>
-  </si>
-  <si>
-    <t>ti lot:</t>
+    <t>Al_ppm</t>
+  </si>
+  <si>
+    <t>%Al</t>
+  </si>
+  <si>
+    <t>al result:</t>
+  </si>
+  <si>
+    <t>al lot:</t>
+  </si>
+  <si>
+    <t>Ca ICP analysis</t>
+  </si>
+  <si>
+    <t>Ca_ppm</t>
+  </si>
+  <si>
+    <t>%Ca</t>
+  </si>
+  <si>
+    <t>ca result:</t>
+  </si>
+  <si>
+    <t>ca oxide factor:</t>
+  </si>
+  <si>
+    <t>ca oxide result:</t>
+  </si>
+  <si>
+    <t>ca lot:</t>
+  </si>
+  <si>
+    <t>Manufacturer: Assurance, 28-35CAY exp: 2026-10-30</t>
   </si>
   <si>
     <t>Note(s):</t>
@@ -138,27 +132,20 @@
     <t>%M+ = [conc.][volume][dilution]/([weight]*10,000)</t>
   </si>
   <si>
-    <t>%Cr(VI) = (1.733[mL FAS][N FAS])/([weight])</t>
-  </si>
-  <si>
-    <t>%Cr2O3 = 1.462*[%Cr(VI)]</t>
-  </si>
-  <si>
-    <t>%Cr(III) = total_Cr - Cr(VI)</t>
+    <t>%MO = [oxide factor]*%M+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.00000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="0.00&quot; ppm&quot;"/>
     <numFmt numFmtId="169" formatCode="0.00&quot; %&quot;"/>
-    <numFmt numFmtId="170" formatCode="0.00"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -236,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -252,9 +239,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -268,7 +252,6 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -576,17 +559,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -594,7 +575,7 @@
         <v>46266</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -602,16 +583,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:3">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="1:5">
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
@@ -619,205 +598,170 @@
         <v>5</v>
       </c>
       <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-    </row>
-    <row r="7" spans="1:5">
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-    </row>
-    <row r="8" spans="1:5">
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-    </row>
-    <row r="9" spans="1:5">
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="B9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="6"/>
+        <v>11</v>
+      </c>
+      <c r="B10" s="7"/>
       <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="11" spans="1:5">
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="C11" s="6"/>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="6">
-        <v>15</v>
-      </c>
-      <c r="B13" s="6">
-        <v>1200</v>
-      </c>
-      <c r="C13" s="6">
-        <v>180</v>
-      </c>
-      <c r="D13" s="6">
-        <v>65</v>
-      </c>
-      <c r="E13" s="6">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="6">
-        <v>15</v>
-      </c>
-      <c r="B14" s="6">
-        <v>1500</v>
-      </c>
-      <c r="C14" s="6">
-        <v>240</v>
-      </c>
-      <c r="D14" s="6">
-        <v>65</v>
-      </c>
-      <c r="E14" s="6">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
       <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-    </row>
-    <row r="16" spans="1:5">
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>18</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="8"/>
+        <v>7</v>
+      </c>
+      <c r="B17" s="6"/>
       <c r="C17" s="6"/>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="6"/>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="6"/>
+        <v>8</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="6"/>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="6"/>
     </row>
     <row r="23" spans="1:3">
-      <c r="A23" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
+      <c r="A23" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="C24" s="6"/>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>18</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" s="8"/>
+        <v>7</v>
+      </c>
+      <c r="B26" s="6"/>
       <c r="C26" s="6"/>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="6"/>
+        <v>8</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="7"/>
+      <c r="C28" s="6"/>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="7"/>
+      <c r="C29" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
+  <mergeCells count="12">
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -825,14 +769,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="15" width="7.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="35" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -853,236 +797,561 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="8">
-        <f>G7</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="10"/>
-      <c r="G7" s="11">
-        <f>digestion_page!B26</f>
+        <v>11</v>
+      </c>
+      <c r="B7" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="9">
+        <f>((C7)*(H7)*(I7))/(G7*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="9">
+        <f>D7/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="10">
+        <f>digestion_page!B10</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="10">
+        <f>digestion_page!C10</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="10">
+        <f>(LEFT(B7,FIND("/",B7)-1)/RIGHT(B7,LEN(B7)-FIND("/", B7)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="8">
-        <f>G8</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="10"/>
-      <c r="G8" s="11">
-        <f>digestion_page!B27</f>
+        <v>12</v>
+      </c>
+      <c r="B8" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9">
+        <f>((C8)*(H8)*(I8))/(G8*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="9">
+        <f>D8/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="10">
+        <f>digestion_page!B11</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="10">
+        <f>digestion_page!C11</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="10">
+        <f>(LEFT(B8,FIND("/",B8)-1)/RIGHT(B8,LEN(B8)-FIND("/", B8)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="3"/>
+      <c r="A10" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="12">
+        <f>AVERAGE(D7:D8)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="12"/>
+      <c r="A11" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="11"/>
       <c r="C11" s="13">
-        <f>AVERAGE(D7:D8)*(10000)*(1/1)</f>
+        <f>AVERAGE(E7:E8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="14">
-        <f>AVERAGE(D7:D8)*(1/1)</f>
-        <v>0</v>
-      </c>
+      <c r="A12" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="3" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B14" s="3"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B16" s="6">
         <f>"1/1"</f>
         <v>0</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="15">
+      <c r="C16" s="8"/>
+      <c r="D16" s="9">
         <f>((C16)*(H16)*(I16))/(G16*1)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="9">
         <f>D16/10000</f>
         <v>0</v>
       </c>
-      <c r="G16" s="11">
-        <f>digestion_page!B17</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="11">
-        <f>digestion_page!C17</f>
-        <v>0</v>
-      </c>
-      <c r="I16" s="11">
+      <c r="G16" s="10">
+        <f>digestion_page!B19</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="10">
+        <f>digestion_page!C19</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="10">
         <f>(LEFT(B16,FIND("/",B16)-1)/RIGHT(B16,LEN(B16)-FIND("/", B16)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="5" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B17" s="6">
         <f>"1/1"</f>
         <v>0</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="15">
+      <c r="C17" s="8"/>
+      <c r="D17" s="9">
         <f>((C17)*(H17)*(I17))/(G17*1)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="9">
         <f>D17/10000</f>
         <v>0</v>
       </c>
-      <c r="G17" s="11">
-        <f>digestion_page!B18</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="11">
-        <f>digestion_page!C18</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="11">
+      <c r="G17" s="10">
+        <f>digestion_page!B20</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="10">
+        <f>digestion_page!C20</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="10">
         <f>(LEFT(B17,FIND("/",B17)-1)/RIGHT(B17,LEN(B17)-FIND("/", B17)))</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="12">
+        <f>AVERAGE(D16:D17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="13">
+        <f>AVERAGE(E16:E17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="3"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="8"/>
+      <c r="D25" s="9">
+        <f>((C25)*(H25)*(I25))/(G25*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="9">
+        <f>D25/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="10">
+        <f>digestion_page!B19</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="10">
+        <f>digestion_page!C19</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="10">
+        <f>(LEFT(B25,FIND("/",B25)-1)/RIGHT(B25,LEN(B25)-FIND("/", B25)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="8"/>
+      <c r="D26" s="9">
+        <f>((C26)*(H26)*(I26))/(G26*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="9">
+        <f>D26/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="10">
+        <f>digestion_page!B20</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="10">
+        <f>digestion_page!C20</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="10">
+        <f>(LEFT(B26,FIND("/",B26)-1)/RIGHT(B26,LEN(B26)-FIND("/", B26)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="11"/>
+      <c r="C28" s="12">
+        <f>AVERAGE(D25:D26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="11"/>
+      <c r="C29" s="13">
+        <f>AVERAGE(E25:E26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="3"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="11"/>
+      <c r="C31" s="13">
+        <f>AVERAGE(E25:E26)*(C30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="3"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="9">
+        <f>((C36)*(H36)*(I36))/(G36*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="9">
+        <f>D36/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="10">
+        <f>digestion_page!B28</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="10">
+        <f>digestion_page!C28</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="10">
+        <f>(LEFT(B36,FIND("/",B36)-1)/RIGHT(B36,LEN(B36)-FIND("/", B36)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="8"/>
+      <c r="D37" s="9">
+        <f>((C37)*(H37)*(I37))/(G37*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="9">
+        <f>D37/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="10">
+        <f>digestion_page!B29</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="10">
+        <f>digestion_page!C29</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="10">
+        <f>(LEFT(B37,FIND("/",B37)-1)/RIGHT(B37,LEN(B37)-FIND("/", B37)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B39" s="11"/>
+      <c r="C39" s="12">
+        <f>AVERAGE(D36:D37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="13">
+        <f>AVERAGE(E36:E37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="11"/>
+      <c r="C41" s="3"/>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="13">
+        <f>AVERAGE(E36:E37)*(C41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B43" s="11"/>
+      <c r="C43" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="B45" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="13">
-        <f>AVERAGE(D16:D17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="14">
-        <f>AVERAGE(E16:E17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="B23" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="25">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:F12"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C23:F25"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="C45:F47"/>
   </mergeCells>
-  <conditionalFormatting sqref="C10">
+  <conditionalFormatting sqref="C12:F12">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(C10))=0</formula>
+      <formula>LEN(TRIM(C12))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21:F21">
     <cfRule type="containsBlanks" dxfId="0" priority="2">
       <formula>LEN(TRIM(C21))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C32:F32">
+    <cfRule type="containsBlanks" dxfId="0" priority="3">
+      <formula>LEN(TRIM(C32))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C43:F43">
+    <cfRule type="containsBlanks" dxfId="0" priority="4">
+      <formula>LEN(TRIM(C43))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1091,35 +1360,25 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="16" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="18" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="18" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" s="18" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>